<commit_message>
Pipeline Driven Prompts matched for apples to apples comparision
</commit_message>
<xml_diff>
--- a/Prompt Design.xlsx
+++ b/Prompt Design.xlsx
@@ -5,6 +5,9 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prompt Designs - Operator Granu" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AF Prompt Designs - Operator" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LG Prompt Designs - MCTS" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prompt Comparison" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pipeline Prompts" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -14,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="10">
     <font>
       <name val="Arial"/>
       <color rgb="FF000000"/>
@@ -36,8 +39,42 @@
       <b val="1"/>
       <color rgb="00FFFFFF"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="00595959"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00000000"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00000000"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="00000000"/>
+      <sz val="9"/>
+    </font>
   </fonts>
-  <fills count="6">
+  <fills count="13">
     <fill>
       <patternFill/>
     </fill>
@@ -64,14 +101,95 @@
         <fgColor rgb="00C6EFCE"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001F4E79"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D6E4F7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F2F2F2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E2EFDA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FCE4D6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D9EAD3"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="6">
     <border/>
+    <border>
+      <left style="thin">
+        <color rgb="00BFBFBF"/>
+      </left>
+      <right style="thin">
+        <color rgb="00BFBFBF"/>
+      </right>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00BFBFBF"/>
+      </bottom>
+    </border>
+    <border>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+    </border>
+    <border>
+      <right style="thin">
+        <color rgb="00BFBFBF"/>
+      </right>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+    </border>
+    <border>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00BFBFBF"/>
+      </bottom>
+    </border>
+    <border>
+      <right style="thin">
+        <color rgb="00BFBFBF"/>
+      </right>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00BFBFBF"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="bottom"/>
     </xf>
@@ -98,6 +216,50 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -5778,4 +5940,1955 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E18"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" style="5" min="1" max="1"/>
+    <col width="36" customWidth="1" style="5" min="2" max="2"/>
+    <col width="72" customWidth="1" style="5" min="3" max="3"/>
+    <col width="60" customWidth="1" style="5" min="4" max="4"/>
+    <col width="26" customWidth="1" style="5" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="6" t="inlineStr">
+        <is>
+          <t>MCTS Component</t>
+        </is>
+      </c>
+      <c r="B1" s="6" t="inlineStr">
+        <is>
+          <t>Section Type</t>
+        </is>
+      </c>
+      <c r="C1" s="6" t="inlineStr">
+        <is>
+          <t>Current/Updated Text Summary</t>
+        </is>
+      </c>
+      <c r="D1" s="6" t="inlineStr">
+        <is>
+          <t>Maps To (Multistep)</t>
+        </is>
+      </c>
+      <c r="E1" s="6" t="inlineStr">
+        <is>
+          <t>Match Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="7" t="inlineStr">
+        <is>
+          <t>mcts_expand</t>
+        </is>
+      </c>
+      <c r="B2" s="7" t="inlineStr">
+        <is>
+          <t>Task Description</t>
+        </is>
+      </c>
+      <c r="C2" s="7" t="inlineStr">
+        <is>
+          <t>You are building a data-pipeline to transform multiple source tables into the target table. Given the current 'Operation History', propose up to k ALTERNATIVE candidates for the SINGLE NEXT operation step, ranked from most to least promising. Each candidate is an INDEPENDENT ALTERNATIVE — NOT sequential. For EVERY candidate specify BOTH operator type AND its full configuration.</t>
+        </is>
+      </c>
+      <c r="D2" s="7" t="inlineStr">
+        <is>
+          <t>get_next_operator_prompt + get_join_prompt + get_group_by_aggregate_prompt (combined into one call)</t>
+        </is>
+      </c>
+      <c r="E2" s="10" t="inlineStr">
+        <is>
+          <t>Identical</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="7" t="inlineStr">
+        <is>
+          <t>mcts_expand</t>
+        </is>
+      </c>
+      <c r="B3" s="7" t="inlineStr">
+        <is>
+          <t>Context fields</t>
+        </is>
+      </c>
+      <c r="C3" s="7" t="inlineStr">
+        <is>
+          <t>Allowed Operations, Operation History, Target Table Name, Target Schema, Target Examples, Source Information, FD Hints (fd_hints), k (number of candidates)</t>
+        </is>
+      </c>
+      <c r="D3" s="7" t="inlineStr">
+        <is>
+          <t>get_next_operator_prompt: target_data_name, target_data_schema, target_samples, source_information, operation_history, allowed_operation_list, hints, fd_hints</t>
+        </is>
+      </c>
+      <c r="E3" s="10" t="inlineStr">
+        <is>
+          <t>Identical</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="7" t="inlineStr">
+        <is>
+          <t>mcts_expand</t>
+        </is>
+      </c>
+      <c r="B4" s="7" t="inlineStr">
+        <is>
+          <t>Config Rules — JOIN</t>
+        </is>
+      </c>
+      <c r="C4" s="7" t="inlineStr">
+        <is>
+          <t>[get_hints_section(JOIN_HINT_IDS, fmt='bullet')]
+Hint IDs: [7,8,9]
++ non-hint line: 'You should only use columns that actually exist in the source tables.'
++ Format: TABLES: [[t1, t2]], COLUMNS: [[t1.col_a, t2.col_b], ...]</t>
+        </is>
+      </c>
+      <c r="D4" s="7" t="inlineStr">
+        <is>
+          <t>get_join_prompt — get_hints_section(JOIN_HINT_IDS, fmt='bullet')</t>
+        </is>
+      </c>
+      <c r="E4" s="9" t="inlineStr">
+        <is>
+          <t>Needs Update → Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="7" t="inlineStr">
+        <is>
+          <t>mcts_expand</t>
+        </is>
+      </c>
+      <c r="B5" s="7" t="inlineStr">
+        <is>
+          <t>Config Rules — UNION</t>
+        </is>
+      </c>
+      <c r="C5" s="7" t="inlineStr">
+        <is>
+          <t>Only union tables with EXACTLY the same column names; do NOT rename. If tables have different schemas, use JOIN instead of UNION.
+Format: TABLES: [table1, table2, table3, ...]</t>
+        </is>
+      </c>
+      <c r="D5" s="7" t="inlineStr">
+        <is>
+          <t>get_union_prompt — similar guidance; no canonical hints for UNION</t>
+        </is>
+      </c>
+      <c r="E5" s="10" t="inlineStr">
+        <is>
+          <t>Identical</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="7" t="inlineStr">
+        <is>
+          <t>mcts_expand</t>
+        </is>
+      </c>
+      <c r="B6" s="7" t="inlineStr">
+        <is>
+          <t>Config Rules — GROUP_BY/AGGREGATE</t>
+        </is>
+      </c>
+      <c r="C6" s="7" t="inlineStr">
+        <is>
+          <t>[get_hints_section(GROUPBY_AGG_HINT_IDS, fmt='bullet')]
+Hint IDs: [10,14,16,17,18,20,21]
++ Format: GROUP_BY: [table.col1, ...], AGGREGATIONS: [COUNT(table.col), SUM(table.col2), ...]</t>
+        </is>
+      </c>
+      <c r="D6" s="7" t="inlineStr">
+        <is>
+          <t>get_group_by_aggregate_prompt — get_hints_section(GROUPBY_AGG_HINT_IDS, fmt='bullet')</t>
+        </is>
+      </c>
+      <c r="E6" s="9" t="inlineStr">
+        <is>
+          <t>Needs Update → Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="7" t="inlineStr">
+        <is>
+          <t>mcts_expand</t>
+        </is>
+      </c>
+      <c r="B7" s="7" t="inlineStr">
+        <is>
+          <t>Config Rules — PIVOT/UNPIVOT, NO_MORE_OPERATION</t>
+        </is>
+      </c>
+      <c r="C7" s="7" t="inlineStr">
+        <is>
+          <t>PIVOT / UNPIVOT — no additional configuration needed. Format: (just the operator line)
+NO_MORE_OPERATION — the pipeline is complete. Format: (just the operator line)</t>
+        </is>
+      </c>
+      <c r="D7" s="7" t="inlineStr">
+        <is>
+          <t>No direct multistep equivalent (multistep issues separate prompts per operator type)</t>
+        </is>
+      </c>
+      <c r="E7" s="8" t="inlineStr">
+        <is>
+          <t>No Multistep Equivalent</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="7" t="inlineStr">
+        <is>
+          <t>mcts_expand</t>
+        </is>
+      </c>
+      <c r="B8" s="7" t="inlineStr">
+        <is>
+          <t>Selection Guidance (Canonical Hints)</t>
+        </is>
+      </c>
+      <c r="C8" s="7" t="inlineStr">
+        <is>
+          <t>[get_hints_section(NEXT_OPERATOR_HINT_IDS, fmt='bullet')]
+Hint IDs: [1,2,3,4,5,6,9,11,16]</t>
+        </is>
+      </c>
+      <c r="D8" s="7" t="inlineStr">
+        <is>
+          <t>get_next_operator_prompt — get_hints_section(NEXT_OPERATOR_HINT_IDS, fmt='bullet')</t>
+        </is>
+      </c>
+      <c r="E8" s="9" t="inlineStr">
+        <is>
+          <t>Needs Update → Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="7" t="inlineStr">
+        <is>
+          <t>mcts_expand</t>
+        </is>
+      </c>
+      <c r="B9" s="7" t="inlineStr">
+        <is>
+          <t>Selection Guidance (MCTS-specific rules)</t>
+        </is>
+      </c>
+      <c r="C9" s="7" t="inlineStr">
+        <is>
+          <t>- If the operation history already covers all needed transformations → propose NO_MORE_OPERATION.
+- Do NOT repeat an operation+configuration already present in the operation history.</t>
+        </is>
+      </c>
+      <c r="D9" s="7" t="inlineStr">
+        <is>
+          <t>No multistep equivalent (MCTS tree-search specific)</t>
+        </is>
+      </c>
+      <c r="E9" s="8" t="inlineStr">
+        <is>
+          <t>No Multistep Equivalent</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="7" t="inlineStr">
+        <is>
+          <t>mcts_expand</t>
+        </is>
+      </c>
+      <c r="B10" s="7" t="inlineStr">
+        <is>
+          <t>Output Format</t>
+        </is>
+      </c>
+      <c r="C10" s="7" t="inlineStr">
+        <is>
+          <t>$CANDIDATE N$ ... $END$ delimited blocks with OPERATOR: &lt;TYPE&gt; + configuration lines. Up to k candidates ranked most-to-least promising.</t>
+        </is>
+      </c>
+      <c r="D10" s="7" t="inlineStr">
+        <is>
+          <t>multistep uses $OPERATOR$ delimited single-answer format</t>
+        </is>
+      </c>
+      <c r="E10" s="8" t="inlineStr">
+        <is>
+          <t>No Multistep Equivalent</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="7" t="inlineStr">
+        <is>
+          <t>mcts_simulate</t>
+        </is>
+      </c>
+      <c r="B11" s="7" t="inlineStr">
+        <is>
+          <t>Task Description</t>
+        </is>
+      </c>
+      <c r="C11" s="7" t="inlineStr">
+        <is>
+          <t>You are generating executable Python code at runtime. Your goal is to convert multiple source tables into the format of the target table.</t>
+        </is>
+      </c>
+      <c r="D11" s="7" t="inlineStr">
+        <is>
+          <t>get_python_script_simple — identical task description</t>
+        </is>
+      </c>
+      <c r="E11" s="10" t="inlineStr">
+        <is>
+          <t>Identical</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="7" t="inlineStr">
+        <is>
+          <t>mcts_simulate</t>
+        </is>
+      </c>
+      <c r="B12" s="7" t="inlineStr">
+        <is>
+          <t>Partial Plan section (MCTS-specific)</t>
+        </is>
+      </c>
+      <c r="C12" s="7" t="inlineStr">
+        <is>
+          <t>Partial Operation Plan (treat this as a STARTING GUIDE, not a fixed sequence). Use operations as a hint for first transformation step(s), then reason about additional steps required to produce the correct target schema.</t>
+        </is>
+      </c>
+      <c r="D12" s="7" t="inlineStr">
+        <is>
+          <t>get_python_script_simple — Operation History used as strict sequence, not a guide</t>
+        </is>
+      </c>
+      <c r="E12" s="8" t="inlineStr">
+        <is>
+          <t>No Multistep Equivalent</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="7" t="inlineStr">
+        <is>
+          <t>mcts_simulate</t>
+        </is>
+      </c>
+      <c r="B13" s="7" t="inlineStr">
+        <is>
+          <t>Context fields</t>
+        </is>
+      </c>
+      <c r="C13" s="7" t="inlineStr">
+        <is>
+          <t>Target Table Name, Target Schema, Target Examples, Source Information (with paths), CSV save path</t>
+        </is>
+      </c>
+      <c r="D13" s="7" t="inlineStr">
+        <is>
+          <t>get_python_script_simple — same fields</t>
+        </is>
+      </c>
+      <c r="E13" s="10" t="inlineStr">
+        <is>
+          <t>Identical</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="7" t="inlineStr">
+        <is>
+          <t>mcts_simulate</t>
+        </is>
+      </c>
+      <c r="B14" s="7" t="inlineStr">
+        <is>
+          <t>Step-by-step thinking (MCTS-specific)</t>
+        </is>
+      </c>
+      <c r="C14" s="7" t="inlineStr">
+        <is>
+          <t>Before writing code, THINK STEP BY STEP about: (a) what partial plan implies for first operation(s), (b) intermediate schema produced, (c) further operations needed, (d) data-type fixes or renames required.</t>
+        </is>
+      </c>
+      <c r="D14" s="7" t="inlineStr">
+        <is>
+          <t>No equivalent in get_python_script_simple</t>
+        </is>
+      </c>
+      <c r="E14" s="8" t="inlineStr">
+        <is>
+          <t>No Multistep Equivalent</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="7" t="inlineStr">
+        <is>
+          <t>mcts_simulate</t>
+        </is>
+      </c>
+      <c r="B15" s="7" t="inlineStr">
+        <is>
+          <t>Plan output block (MCTS-specific)</t>
+        </is>
+      </c>
+      <c r="C15" s="7" t="inlineStr">
+        <is>
+          <t>$PLAN$ ... NO_MORE_OPERATION ... $END_PLAN$ block with one operation per line. Same format as operation history.</t>
+        </is>
+      </c>
+      <c r="D15" s="7" t="inlineStr">
+        <is>
+          <t>No equivalent in get_python_script_simple</t>
+        </is>
+      </c>
+      <c r="E15" s="8" t="inlineStr">
+        <is>
+          <t>No Multistep Equivalent</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="7" t="inlineStr">
+        <is>
+          <t>mcts_simulate</t>
+        </is>
+      </c>
+      <c r="B16" s="7" t="inlineStr">
+        <is>
+          <t>Code generation instruction</t>
+        </is>
+      </c>
+      <c r="C16" s="7" t="inlineStr">
+        <is>
+          <t>Generate Python script implementing COMPLETE transformation from raw source tables to final target CSV. Immediately executable — no placeholders. Quote between ```Python and ```.</t>
+        </is>
+      </c>
+      <c r="D16" s="7" t="inlineStr">
+        <is>
+          <t>get_python_script_simple — identical instruction</t>
+        </is>
+      </c>
+      <c r="E16" s="10" t="inlineStr">
+        <is>
+          <t>Identical</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="7" t="inlineStr">
+        <is>
+          <t>mcts_simulate</t>
+        </is>
+      </c>
+      <c r="B17" s="7" t="inlineStr">
+        <is>
+          <t>Hints (under '══ Hints for Python code generation ══' header)</t>
+        </is>
+      </c>
+      <c r="C17" s="7" t="inlineStr">
+        <is>
+          <t>[get_hints_section(PYTHON_SCRIPT_HINT_IDS, fmt='bullet')]
+Hint IDs: [1,2,3,4,5,10,11,16,17,24,27,28,29,30,31,32]
+Replaces previous: 14-bullet intro list + Hint 1-17 numbered block</t>
+        </is>
+      </c>
+      <c r="D17" s="7" t="inlineStr">
+        <is>
+          <t>get_python_script_simple — get_hints_section(PYTHON_SCRIPT_HINT_IDS, fmt='bullet')</t>
+        </is>
+      </c>
+      <c r="E17" s="9" t="inlineStr">
+        <is>
+          <t>Needs Update → Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="7" t="inlineStr">
+        <is>
+          <t>mcts_simulate</t>
+        </is>
+      </c>
+      <c r="B18" s="7" t="inlineStr">
+        <is>
+          <t>Error feedback</t>
+        </is>
+      </c>
+      <c r="C18" s="7" t="inlineStr">
+        <is>
+          <t>Errors in previous attempts: {error_string}</t>
+        </is>
+      </c>
+      <c r="D18" s="7" t="inlineStr">
+        <is>
+          <t>get_python_script_simple — same error feedback line</t>
+        </is>
+      </c>
+      <c r="E18" s="10" t="inlineStr">
+        <is>
+          <t>Identical</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D47"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="28" customWidth="1" style="5" min="1" max="1"/>
+    <col width="70" customWidth="1" style="5" min="2" max="2"/>
+    <col width="70" customWidth="1" style="5" min="3" max="3"/>
+    <col width="70" customWidth="1" style="5" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1" s="5">
+      <c r="A1" s="11" t="inlineStr">
+        <is>
+          <t>Prompt Design Comparison — Operator Granularity</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="18" customHeight="1" s="5">
+      <c r="A2" s="12" t="inlineStr">
+        <is>
+          <t>Each section shows one operator/step. Columns B-D show the prompt text used by each design for that step. {placeholders} are runtime variables filled from source/target info.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="36" customHeight="1" s="5">
+      <c r="A4" s="13" t="inlineStr">
+        <is>
+          <t>Step / Label</t>
+        </is>
+      </c>
+      <c r="B4" s="13" t="inlineStr">
+        <is>
+          <t>Multi-Step (Sequential CoT)</t>
+        </is>
+      </c>
+      <c r="C4" s="13" t="inlineStr">
+        <is>
+          <t>Agentflow (Operator Granularity)</t>
+        </is>
+      </c>
+      <c r="D4" s="13" t="inlineStr">
+        <is>
+          <t>LangGraph / MCTS</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="22" customHeight="1" s="5">
+      <c r="A5" s="14" t="inlineStr">
+        <is>
+          <t>▶  Planner — Analyze Query   —   One-time: identify required operators and tools from the query before the loop begins</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="30" customHeight="1" s="5">
+      <c r="A6" s="15" t="inlineStr">
+        <is>
+          <t>Source file / function</t>
+        </is>
+      </c>
+      <c r="B6" s="16" t="inlineStr">
+        <is>
+          <t>N/A — no explicit query-analysis step</t>
+        </is>
+      </c>
+      <c r="C6" s="17" t="inlineStr">
+        <is>
+          <t>AgentFlow/.../models/planner.py → _analyze_query_operator()</t>
+        </is>
+      </c>
+      <c r="D6" s="18" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="312" customHeight="1" s="5">
+      <c r="A7" s="19" t="inlineStr">
+        <is>
+          <t>Prompt text</t>
+        </is>
+      </c>
+      <c r="B7" s="20" t="inlineStr">
+        <is>
+          <t>(Not applicable — Multi-Step does not have a separate query-analysis/planner step; it directly calls each prompt in sequence.)</t>
+        </is>
+      </c>
+      <c r="C7" s="21" t="inlineStr">
+        <is>
+          <t>[PLANNER — models/planner.py → _analyze_query_operator()]
+Called ONCE at the start of each solve attempt. Uses llm_engine_fixed (smaller model).
+Returns QueryAnalysis — guides subsequent generate_next_step_operator() calls.
+Task: Analyze the given query to determine necessary skills and tools.
+CRITICAL CONSTRAINT: You can ONLY suggest operations and tools that are in the available tools list. Do NOT suggest operations or tools that are not available.
+Inputs:
+- Query: {question}
+- Available tools: {self.available_tools}
+- Metadata for tools: {self.toolbox_metadata}
+Instructions:
+1. Identify the main objectives in the query.
+2. List ONLY the skills and tools that are actually available in the available tools list.
+3. For each skill and tool, explain how it helps address the query.
+4. If the query requires operations not supported by available tools, explicitly note this limitation.
+5. Note any additional considerations.
+Format your response with a summary of the query, lists of skills and tools with explanations, and a section for additional considerations.
+IMPORTANT: Be brief and precise. Focus ONLY on what can be achieved with the available tools.</t>
+        </is>
+      </c>
+      <c r="D7" s="22" t="inlineStr">
+        <is>
+          <t>(Not applicable — LangGraph/MCTS uses MCTS tree search; there is no separate query-analysis/planner step.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="22" customHeight="1" s="5">
+      <c r="A9" s="14" t="inlineStr">
+        <is>
+          <t>▶  Operator Selection   —   Decide which operator to apply next</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="30" customHeight="1" s="5">
+      <c r="A10" s="15" t="inlineStr">
+        <is>
+          <t>Source file / function</t>
+        </is>
+      </c>
+      <c r="B10" s="16" t="inlineStr">
+        <is>
+          <t>prompts/next_operator_prompt.py → get_next_operator_prompt()</t>
+        </is>
+      </c>
+      <c r="C10" s="17" t="inlineStr">
+        <is>
+          <t>AgentFlow/.../models/planner.py → _generate_next_step_operator()</t>
+        </is>
+      </c>
+      <c r="D10" s="18" t="inlineStr">
+        <is>
+          <t>prompts/mcts_expand.py → get_mcts_expand_prompt() [SELECTION GUIDANCE section]</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="572" customHeight="1" s="5">
+      <c r="A11" s="19" t="inlineStr">
+        <is>
+          <t>Prompt text</t>
+        </is>
+      </c>
+      <c r="B11" s="20" t="inlineStr">
+        <is>
+          <t>query1
+You are generating a data-pipeline to transform multiple source tables to target table and you need to answer "what operation should be performed next?". Take this decision based on "operation history", the schema of the source, target tables, and examples in the target table.
+Allowed Operations: {allowed_operation_list}.
+Operation History: {operation_history}
+1. Target Table Name: {target_data_name}
+2. Target Schema: {target_data_schema}
+3. Target Examples: {target_samples}
+4. Source Information: {source_information}
+{fd_hints}
+{hints[0]}
+[Optional static hints from NEXT_OPERATOR_HINT_IDS]
+- Please answer what operation you should perform next based on "operation history", "source tables" and "target tables" information ("schema" as well as the "examples") in one word.
+- If you feel no more operation is needed further, please return 'NO_MORE_OPERATION'.
+- You should only answer from allowed operations.
+- Try not to repeat operation and it's configuration from the operation history.
+- the final answer should be in $ quotes. i.e. $OPERATOR$</t>
+        </is>
+      </c>
+      <c r="C11" s="21" t="inlineStr">
+        <is>
+          <t>[PLANNER — _generate_next_step_operator()]
+Task: Determine the optimal next step to build the data transformation pipeline operator by operator.
+You are operating at OPERATOR granularity. You configure one operator at a time, incrementally building the pipeline.
+CRITICAL CONSTRAINT: You can ONLY use tools from the available tools list.
+=== OPERATOR TOOLS ===
+- Configure_Join_Operator_Tool: Configure a JOIN between two tables.
+- Configure_Union_Operator_Tool: Configure a UNION (stack) of tables with identical schemas.
+- Configure_GroupBy_Aggregate_Operator_Tool: Configure GROUP BY + aggregation.
+- Add_Pivot_Tool: Configure a PIVOT operation (wide format).
+- Add_Unpivot_Tool: Configure an UNPIVOT (melt) operation (narrow format).
+=== UTILITY TOOLS ===
+- Code_Gen_And_Score_Tool: Generate Python code, execute it, and calculate score.
+- Critique_Pipeline_Tool: Critique pipeline and suggest corrections.
+=== DOMAIN HINTS FOR OPERATOR SELECTION ===
+[Hints from NEXT_OPERATOR_HINT_IDS]
+Context:
+- Query: {question}
+- Query Analysis: {query_analysis}
+- Available Tools: {self.available_tools}
+- Toolbox Metadata: {self.toolbox_metadata}
+- Previous Steps and Their Results: {memory.get_actions()}
+- Current Step: {step_count} of {max_step_count}
+- Remaining Steps: {max_step_count - step_count}
+Instructions:
+1. Review the query, schemas, previous steps, and any score feedback.
+2. Determine which operator to configure next, OR whether to generate/score code, OR whether to critique.
+3. Select the single best tool for this step.
+4. Formulate a specific, achievable sub-goal directly achievable by that tool.
+5. Provide all necessary context.
+Response Format:
+1. Justification: Explain your reasoning and choice of tool.
+2. Context: All information the tool needs.
+3. Sub-Goal: The specific objective for the selected tool.
+4. Tool Name: The exact name from the available tools list.</t>
+        </is>
+      </c>
+      <c r="D11" s="22" t="inlineStr">
+        <is>
+          <t>[Part of mcts_expand.py — SELECTION GUIDANCE section]
+NOTE: In LangGraph/MCTS, operator selection and configuration are a single combined prompt.
+The selection guidance is embedded within the expansion prompt.
+You are generating a data-pipeline to transform multiple source tables to the target table and you need to answer "what operation should be performed next?". Take this decision based on "Operation History", the schema of the source, target tables, and examples in the target table.
+SELECTION GUIDANCE (apply these rules when ranking candidates):
+[Hints from NEXT_OPERATOR_HINT_IDS]
+- If the operation history already covers all needed transformations → propose NO_MORE_OPERATION.
+- Do NOT repeat an operation+configuration already present in the operation history.
+Context provided:
+- Allowed Operations: {allowed_operation_list}
+- Operation History: {operation_history}
+- Target Table Name, Schema, Examples
+- Source Information
+- {fd_hints} (functional-dependency hints)
+Output: Up to {k} ranked candidates, each with BOTH operator type AND full configuration.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="22" customHeight="1" s="5">
+      <c r="A13" s="14" t="inlineStr">
+        <is>
+          <t>▶  JOIN Configuration   —   Determine which tables and columns to join</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="30" customHeight="1" s="5">
+      <c r="A14" s="15" t="inlineStr">
+        <is>
+          <t>Source file / function</t>
+        </is>
+      </c>
+      <c r="B14" s="16" t="inlineStr">
+        <is>
+          <t>prompts/configuration_prompts.py → get_join_prompt()</t>
+        </is>
+      </c>
+      <c r="C14" s="17" t="inlineStr">
+        <is>
+          <t>AgentFlow/.../tools/configure_join_operator/tool.py → get_join_prompt()</t>
+        </is>
+      </c>
+      <c r="D14" s="18" t="inlineStr">
+        <is>
+          <t>prompts/mcts_expand.py → get_mcts_expand_prompt() [JOIN section — combined with selection]</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="338" customHeight="1" s="5">
+      <c r="A15" s="19" t="inlineStr">
+        <is>
+          <t>Prompt text</t>
+        </is>
+      </c>
+      <c r="B15" s="20" t="inlineStr">
+        <is>
+          <t>query1
+You are generating a data-pipeline to transform multiple source tables to target table and you need to answer "what tables should be joined and at which columns?". Take this decision based on "Operation History", "Source" and "Target" (table schema as well as the examples) information.
+Allowed Operations: {allowed_operation_list}.
+1. Target Table Name: {target_data_name}
+2. Target Schema: {target_data_schema}
+3. Target Examples: {target_samples}
+4. Multi Source Information: {source_information}
+5. Operation History: {operation_history}
+-You may use the hint in your decision making process.
+Hint : {hints[0]}
+{fd_hints}
+- Please answer which tables should be joined and at which columns that hasn't appeared yet in "operation history".
+[Optional static hints from JOIN_HINT_IDS]
+- You should only answer from available columns of the source tables.
+- Only return two tables that should be joined and on which columns.
+- Choose tables that contain columns similar to columns in the target tables to be joined.
+- The final answer should be in format of list.
+- The first element of list should be the list of two tables that should be joined.
+- The next elements should be list of two columns on which the join should be perfomed.
+- i.e. [ [table1, table2], [table1.join_column1,table2.join_column1], ...]
+- The final answer list should be within $ quotes strictly. [i.e. $ Final Answer List $]</t>
+        </is>
+      </c>
+      <c r="C15" s="21" t="inlineStr">
+        <is>
+          <t>[Configure_Join_Operator_Tool — get_join_prompt()]
+You are generating a data-pipeline to transform multiple source tables to target table and you need to answer "what tables should be joined and at which columns?". Take this decision based on the transformation case information provided below.
+{transformation_case_info}
+(includes: Target Table Name, Target Schema, Target Examples, Multi Source Information, Operation History)
+- Please answer which tables should be joined and at which columns that hasn't appeared yet in "operation history".
+[Hints from JOIN_HINT_IDS]
+- You should only answer from available columns of the source tables.
+- Only return two tables that should be joined and on which columns.
+- You may use the tables that are generated by the previous actions (e.g., join_result_0, join_result_1, etc.).
+- Choose tables that contain columns similar to columns in the target tables to be joined.
+- The final answer should be in format of list.
+- The first element of list should be the list of two tables that should be joined.
+- The next elements should be list of two columns on which the join should be perfomed.
+- i.e. [ [table1, table2], [table1.join_column1,table2.join_column1], ...]
+- The final answer list should be within $ quotes strictly. [i.e. $ Final Answer List $]</t>
+        </is>
+      </c>
+      <c r="D15" s="22" t="inlineStr">
+        <is>
+          <t>[Part of mcts_expand.py — JOIN configuration section]
+NOTE: LangGraph handles JOIN config within the combined expand prompt. No separate JOIN call.
+JOIN — join two tables on shared columns
+[Hints from JOIN_HINT_IDS]
+  • You should only use columns that actually exist in the source tables.
+  Format:
+    TABLES: [[table1, table2]]
+    COLUMNS: [[table1.col_a, table2.col_b], [table1.col_c, table2.col_d], ...]
+    (one pair per join condition; use multiple pairs for composite keys)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="22" customHeight="1" s="5">
+      <c r="A17" s="14" t="inlineStr">
+        <is>
+          <t>▶  UNION Configuration   —   Determine which tables to stack (same schema)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="30" customHeight="1" s="5">
+      <c r="A18" s="15" t="inlineStr">
+        <is>
+          <t>Source file / function</t>
+        </is>
+      </c>
+      <c r="B18" s="16" t="inlineStr">
+        <is>
+          <t>prompts/configuration_prompts.py → get_union_prompt()</t>
+        </is>
+      </c>
+      <c r="C18" s="17" t="inlineStr">
+        <is>
+          <t>AgentFlow/.../tools/configure_union_operator/tool.py → get_union_prompt()</t>
+        </is>
+      </c>
+      <c r="D18" s="18" t="inlineStr">
+        <is>
+          <t>prompts/mcts_expand.py → get_mcts_expand_prompt() [UNION section — combined with selection]</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="234" customHeight="1" s="5">
+      <c r="A19" s="19" t="inlineStr">
+        <is>
+          <t>Prompt text</t>
+        </is>
+      </c>
+      <c r="B19" s="20" t="inlineStr">
+        <is>
+          <t>You are generating a data-pipeline to transform multiple source tables to target table and you need to answer "what tables should be Union-ed?". Take this decision based on "Operation History",few shot examples, "Source" and "Target" (table schema as well as the examples) information.
+Allowed Operations: {allowed_operation_list}.
+1. Target Table Name: {target_data_name}
+2. Target Schema: {target_data_schema}
+3. Target Examples: {target_samples}
+4. Multi Source Information: {source_information}
+5. Operation History: {operation_history}
+- Please answer which tables should be unioned.
+- Apply UNION to tables that have exactly the same schema without renaming columns.
+- Choose tables having exactly the same schema to union.
+- Try not to repeat operation and it's configuration. i.e. Union on tables should only appear once in "Operation History".
+- You should only answer from available tables of the source tables.
+- Please don't write your reasoning with the answer, just the answer would suffice.
+- The final answer should be in format of list where elements are quoted by $. I.e. [$table1$, $table2$, ...].</t>
+        </is>
+      </c>
+      <c r="C19" s="21" t="inlineStr">
+        <is>
+          <t>[Configure_Union_Operator_Tool — get_union_prompt()]
+You are generating a data-pipeline to transform multiple source tables to target table and you need to answer "what tables should be Union-ed?". Take this decision based on "Operation History",few shot examples, "Source" and "Target" (table schema as well as the examples) information provided below.
+{transformation_case_info}
+(includes: Target Table Name, Target Schema, Target Examples, Multi Source Information, Operation History)
+- Please answer which tables should be unioned.
+- Apply UNION to tables that have exactly the same schema without renaming columns.
+- Choose tables having exactly the same schema to union.
+- Try not to repeat operation and it's configuration. i.e. Union on tables should only appear once in "Operation History".
+- You should only answer from available tables of the source tables.
+- Please don't write your reasoning with the answer, just the answer would suffice.
+- The final answer should be in format of list where elements are quoted by $. I.e. [$table1$, $table2$, ...].</t>
+        </is>
+      </c>
+      <c r="D19" s="22" t="inlineStr">
+        <is>
+          <t>[Part of mcts_expand.py — UNION configuration section]
+NOTE: LangGraph handles UNION config within the combined expand prompt. No separate UNION call.
+UNION — stack tables that have IDENTICAL schemas
+  • Only union tables with EXACTLY the same column names; do NOT rename.
+  • If tables have different schemas, use JOIN instead of UNION.
+  Format:
+    TABLES: [table1, table2, table3, ...]</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="22" customHeight="1" s="5">
+      <c r="A21" s="14" t="inlineStr">
+        <is>
+          <t>▶  GROUP_BY / AGGREGATE Configuration   —   Determine group-by columns, aggregation columns and functions</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="30" customHeight="1" s="5">
+      <c r="A22" s="15" t="inlineStr">
+        <is>
+          <t>Source file / function</t>
+        </is>
+      </c>
+      <c r="B22" s="16" t="inlineStr">
+        <is>
+          <t>prompts/configuration_prompts.py → get_group_by_aggregate_prompt()</t>
+        </is>
+      </c>
+      <c r="C22" s="17" t="inlineStr">
+        <is>
+          <t>AgentFlow/.../tools/configure_group_by_aggregate_operator/tool.py → get_group_by_aggregate_prompt()</t>
+        </is>
+      </c>
+      <c r="D22" s="18" t="inlineStr">
+        <is>
+          <t>prompts/mcts_expand.py → get_mcts_expand_prompt() [GROUP_BY section — combined with selection]</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="273" customHeight="1" s="5">
+      <c r="A23" s="19" t="inlineStr">
+        <is>
+          <t>Prompt text</t>
+        </is>
+      </c>
+      <c r="B23" s="20" t="inlineStr">
+        <is>
+          <t>You are generating a data-pipeline to transform multiple source tables to target table and you need to answer "1. Which columns should be used for Group By operation? 2. Which columns should be Aggregated? 3.Which Aggregation functions should be used?". Take this decision based on "Operation History", few-shot-examples, "Source" and "Target" (table schema as well as the examples) information.
+Allowed Operations: {allowed_operation_list}.
+1. Target Table Name: {target_data_name}
+2. Target Schema: {target_data_schema}
+3. Target Examples: {target_samples}
+4. Multi Source Information: {source_information}
+5. Operation History: {operation_history}
+-You may use the hint in your decision making process.
+Hint : {hints[0]}
+{fd_hints}
+- Please answer on which columns "Group By" operation should be performed, on which columns aggregation should be performed and which aggregation functions should be used.
+[Optional static hints from GROUPBY_AGG_HINT_IDS]
+- You should only answer from available columns of the source tables.
+- Please don't write your reasoning with the answer, just the answer would suffice.
+- The final answer should be in the following format. lists where first list should be group by columns, next list should cover aggregation function and on which columns aggregations should be performed.
+- Example : "group_by" = [table_name.group_by_column1, ...], "aggregations" = [agg_func(table_name.col), ...]</t>
+        </is>
+      </c>
+      <c r="C23" s="21" t="inlineStr">
+        <is>
+          <t>[Configure_GroupBy_Aggregate_Operator_Tool — get_group_by_aggregate_prompt()]
+You are generating a data-pipeline to transform multiple source tables to target table and you need to answer "1. Which columns should be used for Group By operation? 2. Which columns should be Aggregated? 3.Which Aggregation functions should be used?". Take this decision based on the transformation case information provided below.
+{transformation_case_info}
+(includes: Target Table Name, Target Schema, Target Examples, Multi Source Information, Operation History)
+- Please answer on which columns "Group By" operation should be performed, on which columns aggregation should be performed and which aggregation functions should be used.
+[Hints from GROUPBY_AGG_HINT_IDS]
+- You should only answer from available columns of the source tables.
+- Please don't write your reasoning with the answer, just the answer would suffice.
+- The final answer should be in the following format:
+  "group_by" = [table_name.group_by_column1, ...], "aggregations" = [agg_func(table_name.col), ...]</t>
+        </is>
+      </c>
+      <c r="D23" s="22" t="inlineStr">
+        <is>
+          <t>[Part of mcts_expand.py — GROUP_BY/AGGREGATE configuration section]
+NOTE: LangGraph handles GROUP_BY config within the combined expand prompt. No separate call.
+GROUP_BY/AGGREGATE — group rows and apply aggregate functions
+[Hints from GROUPBY_AGG_HINT_IDS]
+  Format:
+    GROUP_BY: [table.col1, table.col2, ...]
+    AGGREGATIONS: [COUNT(table.col), SUM(table.col2), AVG(table.col3), ...]</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="22" customHeight="1" s="5">
+      <c r="A25" s="14" t="inlineStr">
+        <is>
+          <t>▶  PIVOT Configuration   —   Turn row values into column headers (wide format)</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="30" customHeight="1" s="5">
+      <c r="A26" s="15" t="inlineStr">
+        <is>
+          <t>Source file / function</t>
+        </is>
+      </c>
+      <c r="B26" s="16" t="inlineStr">
+        <is>
+          <t>N/A — no dedicated PIVOT prompt</t>
+        </is>
+      </c>
+      <c r="C26" s="17" t="inlineStr">
+        <is>
+          <t>AgentFlow/.../tools/add_pivot/tool.py → get_pivot_prompt()</t>
+        </is>
+      </c>
+      <c r="D26" s="18" t="inlineStr">
+        <is>
+          <t>prompts/mcts_expand.py → PIVOT section (minimal; params resolved at simulation)</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="286" customHeight="1" s="5">
+      <c r="A27" s="19" t="inlineStr">
+        <is>
+          <t>Prompt text</t>
+        </is>
+      </c>
+      <c r="B27" s="20" t="inlineStr">
+        <is>
+          <t>(No dedicated PIVOT prompt in Multi-Step; PIVOT is handled by the code generation prompt after selection)</t>
+        </is>
+      </c>
+      <c r="C27" s="21" t="inlineStr">
+        <is>
+          <t>[Add_Pivot_Tool — get_pivot_prompt()]
+You are configuring a PIVOT operation for a data pipeline that transforms multiple source tables into a target table.
+A PIVOT operation takes rows and turns distinct values from one column into new column headers, aggregating values from another column.
+{transformation_case_info}
+(includes: Target Table Name, Target Schema, Target Examples, Source Information, Operation History)
+Based on the source and target schema information above, determine the correct PIVOT configuration.
+Instructions:
+- Identify the "index" columns: columns kept as row identifiers.
+- Identify the "columns" field: the source column whose distinct values become new column headers.
+- Identify the "values" field: the source column whose values fill the pivoted cells.
+- Identify the "aggfunc": aggregation function ("first", "sum", "mean", "count"). Use "first" if values are unique per cell.
+- The result column names after pivot should match the target schema.
+- You may reference intermediate results from the operation history (e.g., join_result_0).
+Return ONLY the JSON pivot specification enclosed in $ signs:
+${"index": ["col1", "col2"], "columns": "pivot_key_col", "values": "value_col", "aggfunc": "first"}$</t>
+        </is>
+      </c>
+      <c r="D27" s="22" t="inlineStr">
+        <is>
+          <t>[Part of mcts_expand.py — PIVOT/UNPIVOT section]
+NOTE: LangGraph includes PIVOT in the combined expand prompt with minimal config required.
+PIVOT / UNPIVOT — no additional configuration needed
+  Format: (just the operator line; no TABLES or COLUMNS line)
+The LLM selects PIVOT as a candidate operator type. Actual PIVOT parameters
+(index, columns, values, aggfunc) are resolved at code generation time in mcts_simulate.py.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="22" customHeight="1" s="5">
+      <c r="A29" s="14" t="inlineStr">
+        <is>
+          <t>▶  UNPIVOT Configuration   —   Turn column headers into rows (narrow format / melt)</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="30" customHeight="1" s="5">
+      <c r="A30" s="15" t="inlineStr">
+        <is>
+          <t>Source file / function</t>
+        </is>
+      </c>
+      <c r="B30" s="16" t="inlineStr">
+        <is>
+          <t>N/A — no dedicated UNPIVOT prompt</t>
+        </is>
+      </c>
+      <c r="C30" s="17" t="inlineStr">
+        <is>
+          <t>AgentFlow/.../tools/add_unpivot/tool.py → get_unpivot_prompt()</t>
+        </is>
+      </c>
+      <c r="D30" s="18" t="inlineStr">
+        <is>
+          <t>prompts/mcts_expand.py → UNPIVOT section (minimal; params resolved at simulation)</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="247" customHeight="1" s="5">
+      <c r="A31" s="19" t="inlineStr">
+        <is>
+          <t>Prompt text</t>
+        </is>
+      </c>
+      <c r="B31" s="20" t="inlineStr">
+        <is>
+          <t>(No dedicated UNPIVOT prompt in Multi-Step; UNPIVOT is handled by the code generation prompt after selection)</t>
+        </is>
+      </c>
+      <c r="C31" s="21" t="inlineStr">
+        <is>
+          <t>[Add_Unpivot_Tool — get_unpivot_prompt()]
+You are configuring an UNPIVOT (melt) operation for a data pipeline that transforms multiple source tables into a target table.
+An UNPIVOT operation takes a wide table with multiple value columns and stacks those columns into rows, producing a narrower table with a key column and a value column.
+{transformation_case_info}
+(includes: Target Table Name, Target Schema, Target Examples, Source Information, Operation History)
+Instructions:
+- Identify "id_vars": columns to keep as-is (row identifiers that should NOT be melted).
+- Identify "value_vars": columns whose values should be stacked into rows. Leave [] to melt all non-id_vars.
+- Identify "var_name": name for the new column holding the former column names.
+- Identify "value_name": name for the new column holding the values.
+- You may reference intermediate results from the operation history.
+Return ONLY the JSON unpivot specification enclosed in $ signs:
+${"id_vars": ["col1", "col2"], "value_vars": ["col3", "col4"], "var_name": "key_col", "value_name": "val_col"}$</t>
+        </is>
+      </c>
+      <c r="D31" s="22" t="inlineStr">
+        <is>
+          <t>[Part of mcts_expand.py — PIVOT/UNPIVOT section]
+NOTE: LangGraph includes UNPIVOT in the combined expand prompt with minimal config required.
+PIVOT / UNPIVOT — no additional configuration needed
+  Format: (just the operator line; no TABLES or COLUMNS line)
+The LLM selects UNPIVOT as a candidate operator type. Actual UNPIVOT parameters
+(id_vars, value_vars, var_name, value_name) are resolved at code generation time in mcts_simulate.py.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="22" customHeight="1" s="5">
+      <c r="A33" s="14" t="inlineStr">
+        <is>
+          <t>▶  Code Generation   —   Generate executable Python script for the transformation</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="30" customHeight="1" s="5">
+      <c r="A34" s="15" t="inlineStr">
+        <is>
+          <t>Source file / function</t>
+        </is>
+      </c>
+      <c r="B34" s="16" t="inlineStr">
+        <is>
+          <t>prompts/code_generation_prompt.py → get_python_script_simple()</t>
+        </is>
+      </c>
+      <c r="C34" s="17" t="inlineStr">
+        <is>
+          <t>AgentFlow/.../tools/code_gen_and_score/tool.py → get_operator_code_generation_prompt()</t>
+        </is>
+      </c>
+      <c r="D34" s="18" t="inlineStr">
+        <is>
+          <t>prompts/mcts_simulate.py → get_mcts_simulate_prompt()</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="546" customHeight="1" s="5">
+      <c r="A35" s="19" t="inlineStr">
+        <is>
+          <t>Prompt text</t>
+        </is>
+      </c>
+      <c r="B35" s="20" t="inlineStr">
+        <is>
+          <t>You are generating executable Python code at runtime. Please generate a Python script to convert multiple source tables to the format of the target table and STRICTLY follow the sequence of the operations mentioned in 'operation_history' list. The code should immediately executable in a correct way, which means it should NOT contain any placeholder for brievity. For example, even if there exists hundreds of source tables, these data needs to be loaded completely one by one or in a programmable way.
+    Transformation Plan:
+    Operation History: {operation_history}
+    1. Target Table Name: {target_data_name}
+    2. Target Schema: {target_data_schema}
+    3. Target Examples: {target_samples}
+    4. Source Information: {source_information_with_location}
+    5. Write the result to this path {csv_save_path}
+    Based on the transformation plan, generate the Python script that implements the transformation. The script should handle data import, transformation, and export. The script should be complete and executable, not omiting any single statement. For example, please list all the source paths that will be used.
+    Please quote the Python script between one single "```Python" and "```".
+[Optional hints from PYTHON_SCRIPT_HINT_IDS]
+ Errors in previous Attempts : {error_string}</t>
+        </is>
+      </c>
+      <c r="C35" s="21" t="inlineStr">
+        <is>
+          <t>[Code_Gen_And_Score_Tool — get_operator_code_generation_prompt()]
+You are generating executable Python code at runtime. Please generate a Python script to convert multiple source tables to the format of the target table and STRICTLY follow the sequence of the operations mentioned in the action history below. The code should be immediately executable in a correct way, which means it should NOT contain any placeholder for brevity. For example, even if there exist hundreds of source tables, these data need to be loaded completely one by one or in a programmable way.
+    Transformation Context:
+    {query}
+    (includes: Target Table Name, Target Schema, Target Examples, Source Information with file locations, CSV save path)
+    Action History (follow this sequence of operations strictly):
+    {memory_actions}
+    Based on the transformation context and action history, generate the Python script that implements the transformation. The script should handle data import, transformation, and export. The script should be complete and executable, not omitting any single statement.
+    Please quote the Python script between one single "```Python" and "```".
+    Hints to be considered for Python code generation:
+[Hints from PYTHON_SCRIPT_HINT_IDS]
+ Please quote the Python script between one single "```Python" and "```".
+ Errors in previous attempts: {error_string}</t>
+        </is>
+      </c>
+      <c r="D35" s="22" t="inlineStr">
+        <is>
+          <t>[mcts_simulate.py — get_mcts_simulate_prompt()]
+You are generating executable Python code at runtime. Please generate a Python script to convert multiple source tables to the format of the target table. The code should be immediately executable in a correct way, which means it should NOT contain any placeholder for brevity. For example, even if there exist hundreds of source tables, these data need to be loaded completely one by one or in a programmable way.
+Partial Operation Plan (treat this as a STARTING GUIDE, not a fixed sequence):
+{operation_history}
+Use the operations above as a hint for the first transformation step(s), then reason
+about what additional steps are required to produce the correct target schema.
+1. Target Table Name:              {target_data_name}
+2. Target Schema:                  {target_data_schema}
+3. Target Examples:                {target_samples}
+4. Source Information (with paths): {source_information_with_location}
+5. Save the result to:             {csv_save_path}
+Before writing code, THINK STEP BY STEP about the complete transformation plan:
+  a) What does the partial plan above imply for the first operation(s)?
+  b) After those operations, what intermediate schema is produced?
+  c) What further operations are needed to reach the target schema?
+  d) Are there any data-type fixes, string conversions, or column renames required?
+Then output your COMPLETE operation plan using this block (one operation per line,
+ending with NO_MORE_OPERATION):
+$PLAN$
+&lt;operation 1&gt;
+...
+NO_MORE_OPERATION
+$END_PLAN$
+Then generate the Python script that implements the COMPLETE transformation.
+The code must be immediately executable — no placeholders, no ellipses.
+Keep the code brief: no inline comments, no docstrings, no explanatory print statements.
+Please quote the Python script between one single "```Python" and "```".
+Hints for Python code generation:
+[Hints from PYTHON_SCRIPT_HINT_IDS]
+Errors in previous attempts: {error_string}</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="22" customHeight="1" s="5">
+      <c r="A37" s="14" t="inlineStr">
+        <is>
+          <t>▶  Critique — Pipeline Analysis   —   Identify what is wrong with the current pipeline and suggest corrections</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="30" customHeight="1" s="5">
+      <c r="A38" s="15" t="inlineStr">
+        <is>
+          <t>Source file / function</t>
+        </is>
+      </c>
+      <c r="B38" s="16" t="inlineStr">
+        <is>
+          <t>prompts/history_critique.txt (loaded by methods/critique.py)</t>
+        </is>
+      </c>
+      <c r="C38" s="17" t="inlineStr">
+        <is>
+          <t>AgentFlow/.../tools/critique_pipeline/tool.py → get_critique_prompt()</t>
+        </is>
+      </c>
+      <c r="D38" s="18" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="494" customHeight="1" s="5">
+      <c r="A39" s="19" t="inlineStr">
+        <is>
+          <t>Prompt text</t>
+        </is>
+      </c>
+      <c r="B39" s="20" t="inlineStr">
+        <is>
+          <t>[prompts/history_critique.txt — loaded by methods/critique.py]
+You are generating a data-pipeline to transform multiple source tables to follw the schema of the target table. Up to this point, an LLM agent has created a Python Code based on Source Information, Target Information. The python script generated didn't work properly. You will be given Target Data Examples, Functional Dependencies discovered in the Target Table, the operators used in the failed Python code, the schema and the examples of the data generated using the failed Python code.
+Your task is to select operators and configure each operator, and generate Python code based on the list of selected operators.
+--For Join, give the names of tables to be joined and the join attributes;
+--For Union, give the names of tables to be unioned;
+--For GroupBy, give the Group By attributes; You should try group the data by a couple of LEFTMOST column(s) of the given target table schema. These columns often satisfy the following properties: (1) At the leftmost part of the given target table schema; (2) Must be string, or integer types in the source tables or the given target examples and must NOT be float or decimal types; (3) The column must contain unique (non-redundant) values in the given target table examples.
+--For Aggregate, give the aggregation function and aggregation column. Aggregation columns must not be included in group by columns. If many columns in the target table have similar integer values, it probably suggests a count aggregation should be used. If a column (such as X) has float values (such as 1211.2234 or 33.17) in the given target examples, while having integer values (such as 1001 or 35) in the given source tables, it suggests that an "average" aggregation should be applied to X, no matter how X is named. Importantly, this column X MUST BE EXCLUDED from the group by columns.
+--For Filter, give the predicate;
+--For String operators, give a description;
+--It may also contain other operators, such as Complete Table (Add missing rows to the table), Pivot, Next Row (Give the next row).
+Source Data Information: $SRC_INFO$
+Target Data Information :
+Schema :  $SCHEMA$
+Number of Tuples: $NUM_TUPLES$
+Examples : $EXAMPLES$
+Functional Dependencies (FDs) (Important FDs are ranked on top):
+$FD_HINT$
+The failed Python script follow the following operations: $OPERATIONS$
+After these operations, the resulting table that doesn't match target data has schema and examples as follows:
+Schema : $RES_SCHEMA_NOT_AVAILABLE$
+Number of Tuples: $NUM_RES_TUPLES_NOT_AVAILABLE$
+Examples : $RES_EXAMPLES_NOT_AVAILABLE$
+Now you can change those operations to fix the failed transformation. Your code should only take the CSV file paths given in the Source Data Information as inputs. Please make use of all source tables. Do not miss any source table. Please pay attention to the following hints and select relevant hints to apply.
+$STATIC_HINTS$
+[Hints from CRITIQUE_HINT_IDS — injected when static_hints flag is on]
+$METADATA$
+$FEW_SHOT_EXAMPLES$</t>
+        </is>
+      </c>
+      <c r="C39" s="21" t="inlineStr">
+        <is>
+          <t>[Critique_Pipeline_Tool — get_critique_prompt()]
+You are critiquing a data-pipeline that transforms multiple source tables to follow the schema of the target table. An LLM agent has been building this pipeline step by step. Review the current pipeline and suggest corrections.
+Your task is to review the current operation history and suggest what operators need to be changed, added, or removed to correctly produce the target table.
+{transformation_case_info}
+(includes: Target Table Name, Target Schema, Target Examples, Source Information, Operation History)
+For each operator you suggest, provide clear configuration:
+--For Join, give the names of tables to be joined and the join attributes.
+--For Union, give the names of tables to be unioned.
+--For GroupBy, give the Group By attributes. Group by a couple of LEFTMOST column(s) of the target table schema. These columns must be string or integer types (NOT float) and contain unique values in the target examples.
+--For Aggregate, give the aggregation function and aggregation column. Aggregation columns must not be included in group by columns.
+Please pay attention to the following hints and apply relevant ones:
+[Hints from CRITIQUE_HINT_IDS — numbered]
+Based on your analysis, provide:
+1. What is wrong with the current pipeline (if anything).
+2. What specific operators and configurations should be added, changed, or removed.
+3. The corrected sequence of operations.
+Format your response as:
+$CRITIQUE: &lt;your detailed critique and corrected pipeline&gt;$</t>
+        </is>
+      </c>
+      <c r="D39" s="22" t="inlineStr">
+        <is>
+          <t>(Not applicable — LangGraph/MCTS does not have a dedicated critique step. The MCTS tree search explores alternative operator candidates instead of critiquing a fixed pipeline.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="22" customHeight="1" s="5">
+      <c r="A41" s="14" t="inlineStr">
+        <is>
+          <t>▶  Critique — Code Refinement   —   Refine the Python script based on the critique response (Multi-Step only)</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="30" customHeight="1" s="5">
+      <c r="A42" s="15" t="inlineStr">
+        <is>
+          <t>Source file / function</t>
+        </is>
+      </c>
+      <c r="B42" s="16" t="inlineStr">
+        <is>
+          <t>methods/critique.py → query_generator (second LLM call)</t>
+        </is>
+      </c>
+      <c r="C42" s="17" t="inlineStr">
+        <is>
+          <t>N/A — Agentflow critique is a single call; code re-generation is handled by Code_Gen_And_Score_Tool on the next planner step</t>
+        </is>
+      </c>
+      <c r="D42" s="18" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="260" customHeight="1" s="5">
+      <c r="A43" s="19" t="inlineStr">
+        <is>
+          <t>Prompt text</t>
+        </is>
+      </c>
+      <c r="B43" s="20" t="inlineStr">
+        <is>
+          <t>[Second LLM call in methods/critique.py — query_generator]
+NOTE: This is a follow-up call that takes the critique response and refines the Python code.
+Based on the LLM response, can you refine the python code.
+[Optional hints from CRITIQUE_HINT_IDS]
+Note : - Make sure to write the final output of the python code to {target_location_critique}
+    - Make sure to write the python code in-between "```Python" and "```"
+    - Please keep the final output columns the same as it was in the python script given. [Strictly do not add prefix or suffix to the column names]
+    - You just need to apply the fix according to the criticizer response.
+    - Do not use assignment operation for any column.
+    Python Code : ```Python
+    {python_code}
+    ```
+    Code fixing suggestions : ```
+    {res}
+    ```</t>
+        </is>
+      </c>
+      <c r="C43" s="21" t="inlineStr">
+        <is>
+          <t>(No separate code-refinement prompt — the planner invokes Code_Gen_And_Score_Tool again after critique feedback is stored in memory)</t>
+        </is>
+      </c>
+      <c r="D43" s="22" t="inlineStr">
+        <is>
+          <t>(Not applicable — LangGraph/MCTS does not have a dedicated critique step. The MCTS tree search explores alternative operator candidates instead of critiquing a fixed pipeline.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="22" customHeight="1" s="5">
+      <c r="A45" s="14" t="inlineStr">
+        <is>
+          <t>▶  Verifier — STOP / CONTINUE   —   After each tool call: decide whether the pipeline is complete (STOP) or needs more operators/critique (CONTINUE)</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="30" customHeight="1" s="5">
+      <c r="A46" s="15" t="inlineStr">
+        <is>
+          <t>Source file / function</t>
+        </is>
+      </c>
+      <c r="B46" s="16" t="inlineStr">
+        <is>
+          <t>N/A — no verifier; Multi-Step runs a fixed-length sequential loop</t>
+        </is>
+      </c>
+      <c r="C46" s="17" t="inlineStr">
+        <is>
+          <t>AgentFlow/.../models/verifier.py → verificate_context() (non-multimodal)</t>
+        </is>
+      </c>
+      <c r="D46" s="18" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="364" customHeight="1" s="5">
+      <c r="A47" s="19" t="inlineStr">
+        <is>
+          <t>Prompt text</t>
+        </is>
+      </c>
+      <c r="B47" s="20" t="inlineStr">
+        <is>
+          <t>(Not applicable — Multi-Step does not have a verifier. It runs a fixed number of operator-selection → configuration → code-generation cycles.)</t>
+        </is>
+      </c>
+      <c r="C47" s="21" t="inlineStr">
+        <is>
+          <t>[VERIFIER — models/verifier.py → verificate_context() — non-multimodal branch]
+Called after every planner → tool cycle. Uses llm_engine_fixed (smaller model).
+Returns MemoryVerification(analysis, stop_signal) → STOP or CONTINUE.
+Task: Evaluate whether the operator-driven transformation pipeline has produced a correct and complete result, or whether more steps are needed.
+Context:
+- Query: {question}
+- Available Tools: {self.available_tools}
+- Toolbox Metadata: {self.toolbox_metadata}
+- Initial Analysis: {query_analysis}
+- Memory (Tools Used &amp; Results): {memory.get_actions()}
+Instructions:
+1. Review the query, the operator configurations in memory (Join, Union, GroupBy, Pivot, Unpivot), and any code generation results.
+2. Identify whether all necessary operators have been configured to produce the target schema.
+3. Code and Score Check — Look for results from Code_Gen_And_Score_Tool in memory:
+   - score = 1.0 AND score_summary shows no missed functional dependencies, no missed ground-truth keys, and no missed target columns → conclude STOP.
+   - score &lt; 1.0 OR missed items in any category → conclude CONTINUE.
+   - No Code_Gen_And_Score_Tool result in memory yet → conclude CONTINUE.
+   - execution_success = False in the last result → conclude CONTINUE.
+Final Determination:
+- Conclude STOP only when Code_Gen_And_Score_Tool has been run AND score = 1.0 with no missed items.
+- Conclude CONTINUE in all other cases (operators still missing, code not yet generated, score &lt; 1.0, or execution failed).
+IMPORTANT: Keep your response brief (2-3 sentences max). The response must end with either "Conclusion: STOP" or "Conclusion: CONTINUE".</t>
+        </is>
+      </c>
+      <c r="D47" s="22" t="inlineStr">
+        <is>
+          <t>(Not applicable — LangGraph/MCTS determines termination via simulation scores in the MCTS tree; there is no dedicated verifier prompt.)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="13">
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A5:D5"/>
+    <mergeCell ref="A9:D9"/>
+    <mergeCell ref="A17:D17"/>
+    <mergeCell ref="A37:D37"/>
+    <mergeCell ref="A45:D45"/>
+    <mergeCell ref="A21:D21"/>
+    <mergeCell ref="A29:D29"/>
+    <mergeCell ref="A25:D25"/>
+    <mergeCell ref="A41:D41"/>
+    <mergeCell ref="A2:D2"/>
+    <mergeCell ref="A33:D33"/>
+    <mergeCell ref="A13:D13"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D23"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="28" customWidth="1" style="5" min="1" max="1"/>
+    <col width="70" customWidth="1" style="5" min="2" max="2"/>
+    <col width="70" customWidth="1" style="5" min="3" max="3"/>
+    <col width="70" customWidth="1" style="5" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1" s="5">
+      <c r="A1" s="11" t="inlineStr">
+        <is>
+          <t>Prompt Design Comparison — Pipeline Granularity</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="18" customHeight="1" s="5">
+      <c r="A2" s="12" t="inlineStr">
+        <is>
+          <t>Each section shows one pipeline-level step. Multi-Step uses single_step_cot (one combined call). Agentflow has Create_New_Pipeline (design+code) and Refine_Existing_Pipeline (critique+correct). LangGraph/MCTS has no pipeline-level equivalent.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="36" customHeight="1" s="5">
+      <c r="A4" s="13" t="inlineStr">
+        <is>
+          <t>Step / Label</t>
+        </is>
+      </c>
+      <c r="B4" s="13" t="inlineStr">
+        <is>
+          <t>Multi-Step (single_step_cot)</t>
+        </is>
+      </c>
+      <c r="C4" s="13" t="inlineStr">
+        <is>
+          <t>Agentflow — Create_New_Pipeline</t>
+        </is>
+      </c>
+      <c r="D4" s="13" t="inlineStr">
+        <is>
+          <t>Agentflow — Refine_Existing_Pipeline</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="22" customHeight="1" s="5">
+      <c r="A5" s="14" t="inlineStr">
+        <is>
+          <t>▶  Planner — Analyze Query   —   One-time: decide CREATE NEW vs MODIFY EXISTING pipeline before the loop begins</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="30" customHeight="1" s="5">
+      <c r="A6" s="15" t="inlineStr">
+        <is>
+          <t>Source file / function</t>
+        </is>
+      </c>
+      <c r="B6" s="16" t="inlineStr">
+        <is>
+          <t>N/A — single_step_cot makes a direct call without a planning step</t>
+        </is>
+      </c>
+      <c r="C6" s="17" t="inlineStr">
+        <is>
+          <t>AgentFlow/.../models/planner.py → _analyze_query_pipeline()</t>
+        </is>
+      </c>
+      <c r="D6" s="25" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="390" customHeight="1" s="5">
+      <c r="A7" s="19" t="inlineStr">
+        <is>
+          <t>Prompt text</t>
+        </is>
+      </c>
+      <c r="B7" s="20" t="inlineStr">
+        <is>
+          <t>(Not applicable — Multi-Step single_step_cot does not have a planner/verifier loop; it calls the pipeline design+code prompt once per attempt.)</t>
+        </is>
+      </c>
+      <c r="C7" s="21" t="inlineStr">
+        <is>
+          <t>[PLANNER — models/planner.py → _analyze_query_pipeline()]
+Called ONCE at the start. Uses llm_engine_fixed (smaller model).
+Returns QueryAnalysis — decides CREATE NEW vs MODIFY EXISTING pipeline.
+Task: Analyze the given query at a PIPELINE level to determine whether a new data transformation pipeline needs to be created or an existing pipeline should be modified.
+CRITICAL CONSTRAINT: You can ONLY suggest operations and tools that are in the available tools list. Do NOT suggest operations or tools that are not available.
+Inputs:
+- Query: {question}
+- Available tools: {self.available_tools}
+- Metadata for tools: {self.toolbox_metadata}
+Instructions:
+1. Understand the high-level goal of the query — what is the desired end-to-end data transformation?
+2. Determine whether this requires:
+   a) Creating a NEW pipeline from scratch (no existing pipeline addresses this transformation), or
+   b) Modifying an EXISTING pipeline (the transformation is partially addressed and needs adjustments).
+3. Choose the operation sequence to build the target table: which joins, unions, aggregations, etc. steps to apply, in what order.
+4. List ONLY the skills and tools that are actually available in the available tools list.
+5. Note any additional considerations at the pipeline level.
+Format your response with:
+- A concise summary of the query and the target transformation
+- Pipeline decision: CREATE NEW or MODIFY EXISTING (and why)
+- Required skills and relevant tools from the available list
+- Additional considerations
+IMPORTANT: Be brief and precise. Focus on the pipeline-level strategy, NOT individual operator details.</t>
+        </is>
+      </c>
+      <c r="D7" s="26" t="inlineStr">
+        <is>
+          <t>(Not applicable — LangGraph/MCTS operates at operator granularity only via the MCTS tree search; there is no pipeline-level counterpart.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="22" customHeight="1" s="5">
+      <c r="A9" s="14" t="inlineStr">
+        <is>
+          <t>▶  Planner — Next Step Decision   —   At each loop iteration: choose Create_New_Pipeline or Refine_Existing_Pipeline</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="30" customHeight="1" s="5">
+      <c r="A10" s="15" t="inlineStr">
+        <is>
+          <t>Source file / function</t>
+        </is>
+      </c>
+      <c r="B10" s="16" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="C10" s="17" t="inlineStr">
+        <is>
+          <t>AgentFlow/.../models/planner.py → _generate_next_step_pipeline()</t>
+        </is>
+      </c>
+      <c r="D10" s="25" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="585" customHeight="1" s="5">
+      <c r="A11" s="19" t="inlineStr">
+        <is>
+          <t>Prompt text</t>
+        </is>
+      </c>
+      <c r="B11" s="20" t="inlineStr">
+        <is>
+          <t>(Not applicable — Multi-Step single_step_cot does not have a planner loop.)</t>
+        </is>
+      </c>
+      <c r="C11" s="21" t="inlineStr">
+        <is>
+          <t>[PLANNER — models/planner.py → _generate_next_step_pipeline()]
+Called at each loop iteration. Selects Create_New_Pipeline or Refine_Existing_Pipeline.
+Returns NextStep(justification, context, sub_goal, tool_name).
+Task: Determine the optimal next step at a PIPELINE level to address the given query.
+You are operating at a PIPELINE granularity. Instead of picking individual operators one at a time, you should reason about the pipeline as a whole and decide whether to:
+1. Create a new pipeline — Design the full sequence of operations needed to achieve the target transformation.
+2. Modify the existing pipeline — Adjust, add, remove, or reconfigure operations to fix issues or improve correctness.
+CRITICAL CONSTRAINT: You can ONLY use tools from the available tools list. Do NOT suggest operations, sub-goals, or actions that require tools not in this list.
+Context:
+- Query: {question}
+- Query Analysis: {query_analysis}
+- Available Tools (THESE ARE THE ONLY TOOLS YOU CAN USE): {self.available_tools}
+- Toolbox Metadata: {self.toolbox_metadata}
+- Current Step: {step_count} of {max_step_count}
+- Remaining Steps: {max_step_count - step_count}
+- Previous Steps and Their Results: {memory.get_actions()}
+Instructions:
+1. Review the query, the pipeline-level analysis, and all previous steps.
+2. Decide the pipeline-level action:
+   - If a pipeline is in progress, evaluate whether it is on track or needs refinement.
+3. Select the single best tool from the available tools list for the next step.
+4. Formulate a specific, achievable sub-goal for the selected tool.
+5. Provide all necessary context (data, file names, variables) for the tool to function.
+Pipeline-Level Reasoning:
+- Plan the end-to-end transformation from sources to target.
+- When creating a new pipeline, plan the full sequence.
+- When modifying, identify exactly what is wrong and what change will fix it.
+Response Format:
+1. Justification: Explain your pipeline-level reasoning and choice of tool.
+2. Context: Provide all necessary information for the tool.
+3. Sub-Goal: State the specific objective for the tool.
+4. Tool Name: State the exact name of the selected tool (must be from available tools list).
+Rules:
+- Select only ONE tool from the available tools list.
+- The sub-goal must be directly achievable by the selected tool.
+- The response must end with the Context, Sub-Goal, and Tool Name sections in that order, with no extra content.</t>
+        </is>
+      </c>
+      <c r="D11" s="26" t="inlineStr">
+        <is>
+          <t>(Not applicable — LangGraph/MCTS operates at operator granularity only via the MCTS tree search; there is no pipeline-level counterpart.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="22" customHeight="1" s="5">
+      <c r="A13" s="14" t="inlineStr">
+        <is>
+          <t>▶  Create Pipeline (Design + Code)   —   Single LLM call — think through full pipeline plan then generate executable code</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="30" customHeight="1" s="5">
+      <c r="A14" s="15" t="inlineStr">
+        <is>
+          <t>Source file / function</t>
+        </is>
+      </c>
+      <c r="B14" s="16" t="inlineStr">
+        <is>
+          <t>prompts/code_generation_prompt.py → get_python_script_for_single_step_cot()</t>
+        </is>
+      </c>
+      <c r="C14" s="17" t="inlineStr">
+        <is>
+          <t>AgentFlow/.../tools/Create_New_Pipeline/tool.py → get_pipeline_prompt()</t>
+        </is>
+      </c>
+      <c r="D14" s="25" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="338" customHeight="1" s="5">
+      <c r="A15" s="19" t="inlineStr">
+        <is>
+          <t>Prompt text</t>
+        </is>
+      </c>
+      <c r="B15" s="20" t="inlineStr">
+        <is>
+          <t>[prompts/code_generation_prompt.py → get_python_script_for_single_step_cot()]
+You are generating executable Python code at runtime. Please generate a Python script to convert multiple source tables to the format of the target table. The code should immediately executable in a correct way, which means it should NOT contain any placeholder for brievity. For example, even if there exists hundreds of source tables, these data needs to be loaded completely one by one or in a programmable way. Before generating the code, please think step by step about the transformation plan to convert the source tables to the target table.
+    1. Target Table Name: {target_data_name}
+    2. Target Schema: {target_data_schema}
+    3. Target Examples: {target_samples}
+    4. Source Information: {source_information_with_location}
+    5. Write the result to this path {csv_save_path}
+    Based on the transformation plan, generate the Python script that implements the transformation. The script should handle data import, transformation, and export. The script should be complete and executable, not omiting any single statement. For example, please list all the source paths that will be used.
+    Please quote the Python script between one single "```Python" and "```".
+Hints to be considered for Python code generation:
+[Hints from PIPELINE_HINT_IDS — numbered, always included]
+Please quote the Python script between one single "```Python" and "```".
+Errors in previous Attempts : {error_string}</t>
+        </is>
+      </c>
+      <c r="C15" s="21" t="inlineStr">
+        <is>
+          <t>[AgentFlow/.../tools/Create_New_Pipeline/tool.py → get_pipeline_prompt()]
+NOTE: Single LLM call — pipeline design + code generation combined.
+You are generating executable Python code at runtime. Please generate a Python script to convert multiple source tables to the format of the target table. The code must be immediately executable in a correct way, which means it should NOT contain any placeholder for brevity. For example, even if there exist hundreds of source tables, these data need to be loaded completely one by one or in a programmable way. Before generating the code, think step by step about the full transformation plan.
+{transformation_case_info}
+(includes: Target Table Name, Target Schema, Target Examples, Source Information)
+STEP 1 — Think step by step about the full pipeline:
+  a) What operations (JOIN/UNION/GROUP_BY/AGGREGATE/PIVOT/UNPIVOT) are needed and in what order?
+  b) What columns appear in the target but need aggregation from source?
+  c) Are all source tables used?
+STEP 2 — Output the complete pipeline plan:
+$PIPELINE:
+Step 1: &lt;OPERATION_TYPE&gt; - &lt;configuration details&gt;
+Step 2: &lt;OPERATION_TYPE&gt; - &lt;configuration details&gt;
+...
+$
+STEP 3 — Generate the executable Python script implementing the plan above.
+The code must be immediately executable — no placeholders. Load all source CSV files listed in the source information.
+Please quote the Python script between one single "```Python" and "```".
+[Hints from PIPELINE_HINT_IDS — numbered]</t>
+        </is>
+      </c>
+      <c r="D15" s="26" t="inlineStr">
+        <is>
+          <t>(Not applicable — LangGraph/MCTS operates at operator granularity only via the MCTS tree search; there is no pipeline-level counterpart.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="22" customHeight="1" s="5">
+      <c r="A17" s="14" t="inlineStr">
+        <is>
+          <t>▶  Critique + Refine Pipeline   —   Single LLM call — self-analyze current pipeline, produce corrected plan + code</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="30" customHeight="1" s="5">
+      <c r="A18" s="15" t="inlineStr">
+        <is>
+          <t>Source file / function</t>
+        </is>
+      </c>
+      <c r="B18" s="16" t="inlineStr">
+        <is>
+          <t>N/A — no pipeline-level critique/refine in single_step_cot</t>
+        </is>
+      </c>
+      <c r="C18" s="17" t="inlineStr">
+        <is>
+          <t>AgentFlow/.../tools/Refine_Existing_Pipeline/tool.py → get_refine_pipeline_prompt()</t>
+        </is>
+      </c>
+      <c r="D18" s="25" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="416" customHeight="1" s="5">
+      <c r="A19" s="19" t="inlineStr">
+        <is>
+          <t>Prompt text</t>
+        </is>
+      </c>
+      <c r="B19" s="20" t="inlineStr">
+        <is>
+          <t>(Not applicable — Multi-Step single_step_cot does not have a pipeline-level critique/refine step. Critique is at operator level via methods/critique.py.)</t>
+        </is>
+      </c>
+      <c r="C19" s="21" t="inlineStr">
+        <is>
+          <t>[AgentFlow/.../tools/Refine_Existing_Pipeline/tool.py → get_refine_pipeline_prompt()]
+NOTE: Single LLM call — self-contained critique + corrected plan + corrected code.
+You are critiquing a data-pipeline that transforms multiple source tables to follow the schema of the target table. An LLM agent has created this pipeline plan and generated Python code. Review the current pipeline and suggest corrections, then provide the corrected pipeline plan and executable code.
+{transformation_case_info}
+(includes: Target Table Name, Target Schema, Target Examples, Source Information)
+Current Pipeline:
+{current_pipeline}
+[Execution Context if provided — score feedback, error messages, intermediate output]
+Your task:
+1. Identify what is wrong with the current pipeline (if anything).
+2. Specify what steps need to be added, changed, or removed.
+3. Output the CORRECTED pipeline plan.
+4. Generate the executable Python script for the corrected pipeline. The code must be immediately executable — no placeholders.
+[Hints from CRITIQUE_HINT_IDS — numbered]
+Output format:
+$CRITIQUE: &lt;your detailed analysis of what is wrong and what should change&gt;$
+$PIPELINE:
+Step 1: &lt;OPERATION_TYPE&gt; - &lt;configuration details&gt;
+Step 2: &lt;OPERATION_TYPE&gt; - &lt;configuration details&gt;
+...
+$
+Please quote the Python script between one single "```Python" and "```".</t>
+        </is>
+      </c>
+      <c r="D19" s="26" t="inlineStr">
+        <is>
+          <t>(Not applicable — LangGraph/MCTS operates at operator granularity only via the MCTS tree search; there is no pipeline-level counterpart.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="22" customHeight="1" s="5">
+      <c r="A21" s="14" t="inlineStr">
+        <is>
+          <t>▶  Verifier — STOP / CONTINUE   —   After each pipeline tool: decide whether the pipeline is correct (STOP) or needs refinement (CONTINUE)</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="30" customHeight="1" s="5">
+      <c r="A22" s="15" t="inlineStr">
+        <is>
+          <t>Source file / function</t>
+        </is>
+      </c>
+      <c r="B22" s="16" t="inlineStr">
+        <is>
+          <t>N/A — no verifier; single_step_cot runs for a fixed number of attempts</t>
+        </is>
+      </c>
+      <c r="C22" s="17" t="inlineStr">
+        <is>
+          <t>AgentFlow/.../models/verifier.py → verificate_context_pipeline()</t>
+        </is>
+      </c>
+      <c r="D22" s="25" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="455" customHeight="1" s="5">
+      <c r="A23" s="19" t="inlineStr">
+        <is>
+          <t>Prompt text</t>
+        </is>
+      </c>
+      <c r="B23" s="20" t="inlineStr">
+        <is>
+          <t>(Not applicable — Multi-Step single_step_cot does not have a verifier; it reruns the full pipeline prompt on each failed attempt.)</t>
+        </is>
+      </c>
+      <c r="C23" s="21" t="inlineStr">
+        <is>
+          <t>[VERIFIER — models/verifier.py → verificate_context_pipeline()]
+Called after each pipeline tool. Uses llm_engine_fixed (smaller model).
+Returns PipelineVerification(analysis, stop_signal, finalized_pipeline_id) → STOP or CONTINUE.
+Task: Evaluate if the current pipeline is complete and correct enough to produce the target transformation, or if more modifications are needed.
+Context:
+- Query: {question}
+- Available Tools: {self.available_tools}
+- Toolbox Metadata: {self.toolbox_metadata}
+- Initial Analysis: {query_analysis}
+- Memory (Tools Used &amp; Results): {memory.get_actions()}
+Instructions:
+1. Review the query and the pipeline(s) created/modified in memory.
+2. Assess completeness: Does the latest pipeline fully address the target transformation?
+3. Check the critique: If the latest pipeline's critique says CORRECT, the pipeline is likely ready. However, the critique alone is not sufficient — the score must also confirm correctness.
+4. Score Understanding — interpret score_summary from memory:
+   - Functional Dependency Matching: If functional_dependencies.missed is non-empty → add GROUP BY.
+   - Key Matching: If keys.missed_ground_truth_keys is non-empty → add GROUP BY on those columns.
+   - Column Mapping: If column_mappings.missed_target_columns is non-empty → add JOINs.
+   - The pipeline is ONLY correct when ALL three are satisfied: score = 1.0, no missed items.
+5. Score thresholds:
+   - overall_score = 1.0 AND all missed lists empty → recommend STOP.
+   - Any missed item or low score → recommend CONTINUE.
+   - Failed execution → recommend CONTINUE.
+6. If the pipeline is complete and correct, identify the pipeline_id of the finalized pipeline from the memory.
+Final Determination:
+- If pipeline is complete and correct: explain why, provide pipeline_id, conclude STOP.
+- If modifications still needed: explain what's missing or incorrect, conclude CONTINUE.
+IMPORTANT: The response must end with either "Conclusion: STOP" or "Conclusion: CONTINUE".
+If STOP, you MUST include the finalized_pipeline_id with the pipeline_id to finalize.</t>
+        </is>
+      </c>
+      <c r="D23" s="26" t="inlineStr">
+        <is>
+          <t>(Not applicable — LangGraph/MCTS operates at operator granularity only via the MCTS tree search; there is no pipeline-level counterpart.)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="7">
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A5:D5"/>
+    <mergeCell ref="A9:D9"/>
+    <mergeCell ref="A17:D17"/>
+    <mergeCell ref="A21:D21"/>
+    <mergeCell ref="A2:D2"/>
+    <mergeCell ref="A13:D13"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>